<commit_message>
Update to contact details and roles
</commit_message>
<xml_diff>
--- a/files/Spinney_Gantt_v2.xlsx
+++ b/files/Spinney_Gantt_v2.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryan/Documents/GitHub/spinney/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryan/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50FFCF72-77C1-A340-BE9E-D0C4FA8C1F09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB265D92-6A9F-654F-9495-A0B03333EE9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8560" yWindow="1560" windowWidth="29800" windowHeight="20420" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -694,15 +694,9 @@
     <t>07791 528837</t>
   </si>
   <si>
-    <t>larakriek@gmial.com</t>
-  </si>
-  <si>
     <t>07880 688027</t>
   </si>
   <si>
-    <t>neels.kriek@gmial.com</t>
-  </si>
-  <si>
     <t>07851 601499</t>
   </si>
   <si>
@@ -713,6 +707,12 @@
   </si>
   <si>
     <t>01276 488099</t>
+  </si>
+  <si>
+    <t>larakriek@gmail.com</t>
+  </si>
+  <si>
+    <t>neels.kriek@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -3205,7 +3205,7 @@
         <v>217</v>
       </c>
       <c r="E6" s="28" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3219,10 +3219,10 @@
         <v>29</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E7" s="28" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3236,10 +3236,10 @@
         <v>29</v>
       </c>
       <c r="D8" s="27" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="E8" s="28" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3250,7 +3250,7 @@
         <v>180</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27"/>
@@ -3263,7 +3263,7 @@
         <v>182</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D10" s="27"/>
       <c r="E10" s="27"/>
@@ -3276,7 +3276,7 @@
         <v>182</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D11" s="27"/>
       <c r="E11" s="27"/>
@@ -3289,7 +3289,7 @@
         <v>182</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D12" s="27"/>
       <c r="E12" s="27"/>
@@ -3302,7 +3302,7 @@
         <v>185</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D13" s="27"/>
       <c r="E13" s="27"/>
@@ -3318,7 +3318,7 @@
         <v>43</v>
       </c>
       <c r="D14" s="27" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E14" s="27"/>
     </row>

</xml_diff>